<commit_message>
Atchison Web 11 July v1
</commit_message>
<xml_diff>
--- a/AtchisonRegime/Outputs/Aust/df_regCLI_Aust.xlsx
+++ b/AtchisonRegime/Outputs/Aust/df_regCLI_Aust.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H678"/>
+  <dimension ref="A1:H679"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17797,22 +17797,22 @@
         <v>45504</v>
       </c>
       <c r="B668" t="n">
-        <v>99.74919</v>
+        <v>99.69</v>
       </c>
       <c r="C668" t="n">
-        <v>99.57156000000002</v>
+        <v>99.55183</v>
       </c>
       <c r="D668" t="n">
-        <v>99.76596499999999</v>
+        <v>99.76432083333333</v>
       </c>
       <c r="E668" t="n">
-        <v>0.7902620670330979</v>
+        <v>0.7903595325288878</v>
       </c>
       <c r="F668" t="b">
         <v>1</v>
       </c>
       <c r="G668" t="n">
-        <v>0.2333656234980073</v>
+        <v>0.1584468774600688</v>
       </c>
       <c r="H668" t="b">
         <v>1</v>
@@ -17823,22 +17823,22 @@
         <v>45535</v>
       </c>
       <c r="B669" t="n">
-        <v>99.89503999999999</v>
+        <v>99.83</v>
       </c>
       <c r="C669" t="n">
-        <v>99.73633333333332</v>
+        <v>99.69492333333334</v>
       </c>
       <c r="D669" t="n">
-        <v>99.72754944444445</v>
+        <v>99.72409861111112</v>
       </c>
       <c r="E669" t="n">
-        <v>0.7470949078815513</v>
+        <v>0.7467689263684245</v>
       </c>
       <c r="F669" t="b">
         <v>1</v>
       </c>
       <c r="G669" t="n">
-        <v>0.1952228538320057</v>
+        <v>0.1874743244618221</v>
       </c>
       <c r="H669" t="b">
         <v>1</v>
@@ -17849,22 +17849,22 @@
         <v>45565</v>
       </c>
       <c r="B670" t="n">
-        <v>99.9945</v>
+        <v>99.92</v>
       </c>
       <c r="C670" t="n">
-        <v>99.87957666666667</v>
+        <v>99.81333333333333</v>
       </c>
       <c r="D670" t="n">
-        <v>99.69770777777778</v>
+        <v>99.69218749999999</v>
       </c>
       <c r="E670" t="n">
-        <v>0.7126515616689667</v>
+        <v>0.7113715138092738</v>
       </c>
       <c r="F670" t="b">
         <v>1</v>
       </c>
       <c r="G670" t="n">
-        <v>0.1395632948127991</v>
+        <v>0.1265161708796416</v>
       </c>
       <c r="H670" t="b">
         <v>1</v>
@@ -17875,22 +17875,22 @@
         <v>45596</v>
       </c>
       <c r="B671" t="n">
-        <v>100.0541</v>
+        <v>99.98</v>
       </c>
       <c r="C671" t="n">
-        <v>99.98121333333334</v>
+        <v>99.91000000000001</v>
       </c>
       <c r="D671" t="n">
-        <v>99.6753188888889</v>
+        <v>99.66774027777778</v>
       </c>
       <c r="E671" t="n">
-        <v>0.6872999550114536</v>
+        <v>0.6847112112895861</v>
       </c>
       <c r="F671" t="b">
         <v>1</v>
       </c>
       <c r="G671" t="n">
-        <v>0.08671614127926139</v>
+        <v>0.08762818398576852</v>
       </c>
       <c r="H671" t="b">
         <v>1</v>
@@ -17901,22 +17901,22 @@
         <v>45626</v>
       </c>
       <c r="B672" t="n">
-        <v>100.0893</v>
+        <v>100.02</v>
       </c>
       <c r="C672" t="n">
-        <v>100.0459666666667</v>
+        <v>99.97333333333334</v>
       </c>
       <c r="D672" t="n">
-        <v>99.65849944444443</v>
+        <v>99.64899583333333</v>
       </c>
       <c r="E672" t="n">
-        <v>0.668798441479506</v>
+        <v>0.6647366178328665</v>
       </c>
       <c r="F672" t="b">
         <v>1</v>
       </c>
       <c r="G672" t="n">
-        <v>0.05263170159625388</v>
+        <v>0.06017420874209937</v>
       </c>
       <c r="H672" t="b">
         <v>1</v>
@@ -17927,22 +17927,22 @@
         <v>45657</v>
       </c>
       <c r="B673" t="n">
-        <v>100.1283</v>
+        <v>100.05</v>
       </c>
       <c r="C673" t="n">
-        <v>100.0905666666667</v>
+        <v>100.0166666666667</v>
       </c>
       <c r="D673" t="n">
-        <v>99.64568</v>
+        <v>99.63400138888888</v>
       </c>
       <c r="E673" t="n">
-        <v>0.6547119999336849</v>
+        <v>0.648805822781503</v>
       </c>
       <c r="F673" t="b">
         <v>1</v>
       </c>
       <c r="G673" t="n">
-        <v>0.05956817654778246</v>
+        <v>0.0462387958717568</v>
       </c>
       <c r="H673" t="b">
         <v>1</v>
@@ -17953,22 +17953,22 @@
         <v>45688</v>
       </c>
       <c r="B674" t="n">
-        <v>100.1812</v>
+        <v>100.08</v>
       </c>
       <c r="C674" t="n">
-        <v>100.1329333333333</v>
+        <v>100.05</v>
       </c>
       <c r="D674" t="n">
-        <v>99.63578000000001</v>
+        <v>99.62129027777777</v>
       </c>
       <c r="E674" t="n">
-        <v>0.6434373123867262</v>
+        <v>0.6349313248645349</v>
       </c>
       <c r="F674" t="b">
         <v>1</v>
       </c>
       <c r="G674" t="n">
-        <v>0.08221469128637288</v>
+        <v>0.04724920448113307</v>
       </c>
       <c r="H674" t="b">
         <v>1</v>
@@ -17979,22 +17979,22 @@
         <v>45716</v>
       </c>
       <c r="B675" t="n">
-        <v>100.2467</v>
+        <v>100.11</v>
       </c>
       <c r="C675" t="n">
-        <v>100.1854</v>
+        <v>100.08</v>
       </c>
       <c r="D675" t="n">
-        <v>99.62804111111112</v>
+        <v>99.60975416666666</v>
       </c>
       <c r="E675" t="n">
-        <v>0.6340398023909066</v>
+        <v>0.6216713698473547</v>
       </c>
       <c r="F675" t="b">
         <v>1</v>
       </c>
       <c r="G675" t="n">
-        <v>0.1033058173209403</v>
+        <v>0.04825700756875347</v>
       </c>
       <c r="H675" t="b">
         <v>1</v>
@@ -18005,22 +18005,22 @@
         <v>45747</v>
       </c>
       <c r="B676" t="n">
-        <v>100.3279</v>
+        <v>100.14</v>
       </c>
       <c r="C676" t="n">
-        <v>100.2519333333333</v>
+        <v>100.11</v>
       </c>
       <c r="D676" t="n">
-        <v>99.62204944444444</v>
+        <v>99.59854305555555</v>
       </c>
       <c r="E676" t="n">
-        <v>0.6261101789938501</v>
+        <v>0.6078346349828332</v>
       </c>
       <c r="F676" t="b">
         <v>1</v>
       </c>
       <c r="G676" t="n">
-        <v>0.1296896340680529</v>
+        <v>0.04935552907551643</v>
       </c>
       <c r="H676" t="b">
         <v>1</v>
@@ -18031,22 +18031,22 @@
         <v>45777</v>
       </c>
       <c r="B677" t="n">
-        <v>100.4102</v>
+        <v>100.19</v>
       </c>
       <c r="C677" t="n">
-        <v>100.3282666666667</v>
+        <v>100.1466666666667</v>
       </c>
       <c r="D677" t="n">
-        <v>99.61747444444444</v>
+        <v>99.58785138888888</v>
       </c>
       <c r="E677" t="n">
-        <v>0.6195157575048882</v>
+        <v>0.5933834278015171</v>
       </c>
       <c r="F677" t="b">
         <v>1</v>
       </c>
       <c r="G677" t="n">
-        <v>0.1328456927899113</v>
+        <v>0.08426254872881592</v>
       </c>
       <c r="H677" t="b">
         <v>1</v>
@@ -18057,24 +18057,50 @@
         <v>45808</v>
       </c>
       <c r="B678" t="n">
-        <v>100.5006</v>
+        <v>100.25</v>
       </c>
       <c r="C678" t="n">
-        <v>100.4129</v>
+        <v>100.1933333333333</v>
       </c>
       <c r="D678" t="n">
-        <v>99.61492166666667</v>
+        <v>99.5783375</v>
       </c>
       <c r="E678" t="n">
-        <v>0.6155599865279717</v>
+        <v>0.5793962295374195</v>
       </c>
       <c r="F678" t="b">
         <v>1</v>
       </c>
       <c r="G678" t="n">
-        <v>0.1468581486426662</v>
+        <v>0.1035560760343665</v>
       </c>
       <c r="H678" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="2" t="n">
+        <v>45838</v>
+      </c>
+      <c r="B679" t="n">
+        <v>100.33</v>
+      </c>
+      <c r="C679" t="n">
+        <v>100.2566666666667</v>
+      </c>
+      <c r="D679" t="n">
+        <v>99.57139583333333</v>
+      </c>
+      <c r="E679" t="n">
+        <v>0.5684473597459838</v>
+      </c>
+      <c r="F679" t="b">
+        <v>1</v>
+      </c>
+      <c r="G679" t="n">
+        <v>0.1407342274150892</v>
+      </c>
+      <c r="H679" t="b">
         <v>1</v>
       </c>
     </row>
@@ -18359,13 +18385,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84C0C125-5D1E-4DD3-8EA0-B525FC34CA1A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CFA7E57-D3EB-415E-9E68-083B40765C28}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D825304F-AEEC-47FC-835B-443872433A1A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB6CA3D4-95F0-44FD-B1DB-4B30898E6545}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1796A7A-A571-4E87-944D-572D6AF27443}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F1FFB45-E838-4A66-8958-1418980AEC02}"/>
 </file>
</xml_diff>

<commit_message>
Main Web 30 Sep v1
</commit_message>
<xml_diff>
--- a/AtchisonRegime/Outputs/Aust/df_regCLI_Aust.xlsx
+++ b/AtchisonRegime/Outputs/Aust/df_regCLI_Aust.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H679"/>
+  <dimension ref="A1:H682"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17823,22 +17823,22 @@
         <v>45535</v>
       </c>
       <c r="B669" t="n">
-        <v>99.83</v>
+        <v>99.80953</v>
       </c>
       <c r="C669" t="n">
-        <v>99.69492333333334</v>
+        <v>99.68810000000001</v>
       </c>
       <c r="D669" t="n">
-        <v>99.72409861111112</v>
+        <v>99.72353000000001</v>
       </c>
       <c r="E669" t="n">
-        <v>0.7467689263684245</v>
+        <v>0.7466937755810166</v>
       </c>
       <c r="F669" t="b">
         <v>1</v>
       </c>
       <c r="G669" t="n">
-        <v>0.1874743244618221</v>
+        <v>0.1600790095069279</v>
       </c>
       <c r="H669" t="b">
         <v>1</v>
@@ -17849,22 +17849,22 @@
         <v>45565</v>
       </c>
       <c r="B670" t="n">
-        <v>99.92</v>
+        <v>99.93568</v>
       </c>
       <c r="C670" t="n">
-        <v>99.81333333333333</v>
+        <v>99.81173666666666</v>
       </c>
       <c r="D670" t="n">
-        <v>99.69218749999999</v>
+        <v>99.69205444444444</v>
       </c>
       <c r="E670" t="n">
-        <v>0.7113715138092738</v>
+        <v>0.7114150180207116</v>
       </c>
       <c r="F670" t="b">
         <v>1</v>
       </c>
       <c r="G670" t="n">
-        <v>0.1265161708796416</v>
+        <v>0.1773226552779029</v>
       </c>
       <c r="H670" t="b">
         <v>1</v>
@@ -17875,22 +17875,22 @@
         <v>45596</v>
       </c>
       <c r="B671" t="n">
-        <v>99.98</v>
+        <v>99.99481</v>
       </c>
       <c r="C671" t="n">
-        <v>99.91000000000001</v>
+        <v>99.91334000000001</v>
       </c>
       <c r="D671" t="n">
-        <v>99.66774027777778</v>
+        <v>99.66801861111111</v>
       </c>
       <c r="E671" t="n">
-        <v>0.6847112112895861</v>
+        <v>0.684948986956196</v>
       </c>
       <c r="F671" t="b">
         <v>1</v>
       </c>
       <c r="G671" t="n">
-        <v>0.08762818398576852</v>
+        <v>0.08632759683718989</v>
       </c>
       <c r="H671" t="b">
         <v>1</v>
@@ -17901,22 +17901,22 @@
         <v>45626</v>
       </c>
       <c r="B672" t="n">
-        <v>100.02</v>
+        <v>100.0343</v>
       </c>
       <c r="C672" t="n">
-        <v>99.97333333333334</v>
+        <v>99.98826333333334</v>
       </c>
       <c r="D672" t="n">
-        <v>99.64899583333333</v>
+        <v>99.64967138888889</v>
       </c>
       <c r="E672" t="n">
-        <v>0.6647366178328665</v>
+        <v>0.6652216109931508</v>
       </c>
       <c r="F672" t="b">
         <v>1</v>
       </c>
       <c r="G672" t="n">
-        <v>0.06017420874209937</v>
+        <v>0.05936367572461095</v>
       </c>
       <c r="H672" t="b">
         <v>1</v>
@@ -17927,22 +17927,22 @@
         <v>45657</v>
       </c>
       <c r="B673" t="n">
-        <v>100.05</v>
+        <v>100.0664</v>
       </c>
       <c r="C673" t="n">
-        <v>100.0166666666667</v>
+        <v>100.0318366666667</v>
       </c>
       <c r="D673" t="n">
-        <v>99.63400138888888</v>
+        <v>99.6351325</v>
       </c>
       <c r="E673" t="n">
-        <v>0.648805822781503</v>
+        <v>0.6496241547689788</v>
       </c>
       <c r="F673" t="b">
         <v>1</v>
       </c>
       <c r="G673" t="n">
-        <v>0.0462387958717568</v>
+        <v>0.0494131872473481</v>
       </c>
       <c r="H673" t="b">
         <v>1</v>
@@ -17953,22 +17953,22 @@
         <v>45688</v>
       </c>
       <c r="B674" t="n">
-        <v>100.08</v>
+        <v>100.0915</v>
       </c>
       <c r="C674" t="n">
-        <v>100.05</v>
+        <v>100.0640666666666</v>
       </c>
       <c r="D674" t="n">
-        <v>99.62129027777777</v>
+        <v>99.62274083333334</v>
       </c>
       <c r="E674" t="n">
-        <v>0.6349313248645349</v>
+        <v>0.6360300929555354</v>
       </c>
       <c r="F674" t="b">
         <v>1</v>
       </c>
       <c r="G674" t="n">
-        <v>0.04724920448113307</v>
+        <v>0.03946354154936113</v>
       </c>
       <c r="H674" t="b">
         <v>1</v>
@@ -17979,22 +17979,22 @@
         <v>45716</v>
       </c>
       <c r="B675" t="n">
-        <v>100.11</v>
+        <v>100.1063</v>
       </c>
       <c r="C675" t="n">
-        <v>100.08</v>
+        <v>100.0880666666667</v>
       </c>
       <c r="D675" t="n">
-        <v>99.60975416666666</v>
+        <v>99.61110194444444</v>
       </c>
       <c r="E675" t="n">
-        <v>0.6216713698473547</v>
+        <v>0.6227368050781948</v>
       </c>
       <c r="F675" t="b">
         <v>1</v>
       </c>
       <c r="G675" t="n">
-        <v>0.04825700756875347</v>
+        <v>0.02376605956050688</v>
       </c>
       <c r="H675" t="b">
         <v>1</v>
@@ -18005,22 +18005,22 @@
         <v>45747</v>
       </c>
       <c r="B676" t="n">
-        <v>100.14</v>
+        <v>100.1203</v>
       </c>
       <c r="C676" t="n">
-        <v>100.11</v>
+        <v>100.1060333333333</v>
       </c>
       <c r="D676" t="n">
-        <v>99.59854305555555</v>
+        <v>99.59934361111111</v>
       </c>
       <c r="E676" t="n">
-        <v>0.6078346349828332</v>
+        <v>0.6084592304133375</v>
       </c>
       <c r="F676" t="b">
         <v>1</v>
       </c>
       <c r="G676" t="n">
-        <v>0.04935552907551643</v>
+        <v>0.02300893683622046</v>
       </c>
       <c r="H676" t="b">
         <v>1</v>
@@ -18031,22 +18031,22 @@
         <v>45777</v>
       </c>
       <c r="B677" t="n">
-        <v>100.19</v>
+        <v>100.1385</v>
       </c>
       <c r="C677" t="n">
-        <v>100.1466666666667</v>
+        <v>100.1217</v>
       </c>
       <c r="D677" t="n">
-        <v>99.58785138888888</v>
+        <v>99.58722138888888</v>
       </c>
       <c r="E677" t="n">
-        <v>0.5933834278015171</v>
+        <v>0.5926087949212792</v>
       </c>
       <c r="F677" t="b">
         <v>1</v>
       </c>
       <c r="G677" t="n">
-        <v>0.08426254872881592</v>
+        <v>0.0307116602992886</v>
       </c>
       <c r="H677" t="b">
         <v>1</v>
@@ -18057,22 +18057,22 @@
         <v>45808</v>
       </c>
       <c r="B678" t="n">
-        <v>100.25</v>
+        <v>100.1695</v>
       </c>
       <c r="C678" t="n">
-        <v>100.1933333333333</v>
+        <v>100.1427666666667</v>
       </c>
       <c r="D678" t="n">
-        <v>99.5783375</v>
+        <v>99.57547138888889</v>
       </c>
       <c r="E678" t="n">
-        <v>0.5793962295374195</v>
+        <v>0.5760697993083793</v>
       </c>
       <c r="F678" t="b">
         <v>1</v>
       </c>
       <c r="G678" t="n">
-        <v>0.1035560760343665</v>
+        <v>0.05381292342911231</v>
       </c>
       <c r="H678" t="b">
         <v>1</v>
@@ -18083,24 +18083,102 @@
         <v>45838</v>
       </c>
       <c r="B679" t="n">
-        <v>100.33</v>
+        <v>100.2179</v>
       </c>
       <c r="C679" t="n">
-        <v>100.2566666666667</v>
+        <v>100.1753</v>
       </c>
       <c r="D679" t="n">
-        <v>99.57139583333333</v>
+        <v>99.56541583333333</v>
       </c>
       <c r="E679" t="n">
-        <v>0.5684473597459838</v>
+        <v>0.5609983970712116</v>
       </c>
       <c r="F679" t="b">
         <v>1</v>
       </c>
       <c r="G679" t="n">
-        <v>0.1407342274150892</v>
+        <v>0.0862747563142451</v>
       </c>
       <c r="H679" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="2" t="n">
+        <v>45869</v>
+      </c>
+      <c r="B680" t="n">
+        <v>100.2731</v>
+      </c>
+      <c r="C680" t="n">
+        <v>100.2201666666667</v>
+      </c>
+      <c r="D680" t="n">
+        <v>99.55833805555555</v>
+      </c>
+      <c r="E680" t="n">
+        <v>0.5500080452389596</v>
+      </c>
+      <c r="F680" t="b">
+        <v>1</v>
+      </c>
+      <c r="G680" t="n">
+        <v>0.1003621682952233</v>
+      </c>
+      <c r="H680" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="2" t="n">
+        <v>45900</v>
+      </c>
+      <c r="B681" t="n">
+        <v>100.3164</v>
+      </c>
+      <c r="C681" t="n">
+        <v>100.2691333333333</v>
+      </c>
+      <c r="D681" t="n">
+        <v>99.55528805555555</v>
+      </c>
+      <c r="E681" t="n">
+        <v>0.5453425767603173</v>
+      </c>
+      <c r="F681" t="b">
+        <v>1</v>
+      </c>
+      <c r="G681" t="n">
+        <v>0.07939963216741985</v>
+      </c>
+      <c r="H681" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="2" t="n">
+        <v>45930</v>
+      </c>
+      <c r="B682" t="n">
+        <v>100.3656</v>
+      </c>
+      <c r="C682" t="n">
+        <v>100.3183666666667</v>
+      </c>
+      <c r="D682" t="n">
+        <v>99.55828527777777</v>
+      </c>
+      <c r="E682" t="n">
+        <v>0.5495933020567819</v>
+      </c>
+      <c r="F682" t="b">
+        <v>1</v>
+      </c>
+      <c r="G682" t="n">
+        <v>0.08952074163908909</v>
+      </c>
+      <c r="H682" t="b">
         <v>1</v>
       </c>
     </row>
@@ -18385,13 +18463,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CFA7E57-D3EB-415E-9E68-083B40765C28}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FDE273D-216E-4A80-8318-12C7FDDF0ADE}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB6CA3D4-95F0-44FD-B1DB-4B30898E6545}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E05BE203-86F6-4CA6-A3F0-1A1D425C6CE3}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F1FFB45-E838-4A66-8958-1418980AEC02}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74BC9DE6-F927-4F66-BAD9-8662ED2EF3EC}"/>
 </file>
</xml_diff>